<commit_message>
Code after Regression execution on 26th March'25
</commit_message>
<xml_diff>
--- a/Data/Copy of testDataCzechiaMK_DryRun2.xlsx
+++ b/Data/Copy of testDataCzechiaMK_DryRun2.xlsx
@@ -1,15 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{9EC13EC6-489B-4C00-951D-46CAAC619E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -286,7 +301,7 @@
     <t>Permanent</t>
   </si>
   <si>
-    <t xml:space="preserve">Store Manager_NEW </t>
+    <t>Store Manager_NEW </t>
   </si>
   <si>
     <t>Full Time</t>
@@ -310,7 +325,7 @@
     <t>92 Retail Management</t>
   </si>
   <si>
-    <t xml:space="preserve">251 Management Retail  </t>
+    <t>251 Management Retail  </t>
   </si>
   <si>
     <t>Personal Number</t>
@@ -957,7 +972,7 @@
     <t>Auto 23560374</t>
   </si>
   <si>
-    <t xml:space="preserve">In-Store P&amp;C Manager_NEW </t>
+    <t>In-Store P&amp;C Manager_NEW </t>
   </si>
   <si>
     <t>Test_7</t>
@@ -1578,7 +1593,7 @@
     <t>Auto 11582787</t>
   </si>
   <si>
-    <t xml:space="preserve">Assistant Store Manager_NEW </t>
+    <t>Assistant Store Manager_NEW </t>
   </si>
   <si>
     <t>Test_11</t>
@@ -2152,7 +2167,7 @@
     <t>Auto 28550845</t>
   </si>
   <si>
-    <t xml:space="preserve">Department Manager_NEW </t>
+    <t>Department Manager_NEW </t>
   </si>
   <si>
     <t>Test_15</t>
@@ -2190,7 +2205,7 @@
     <t>TMOneQ</t>
   </si>
   <si>
-    <t xml:space="preserve">Team Manager - Retail_NEW </t>
+    <t>Team Manager - Retail_NEW </t>
   </si>
   <si>
     <t>Test_19</t>
@@ -2220,7 +2235,7 @@
     <t>Auto 26102024 181953</t>
   </si>
   <si>
-    <t xml:space="preserve">In-Store P&amp;C Supervisor_NEW </t>
+    <t>In-Store P&amp;C Supervisor_NEW </t>
   </si>
   <si>
     <t>Test_23</t>
@@ -2250,7 +2265,7 @@
     <t>Auto 26102024 185305</t>
   </si>
   <si>
-    <t xml:space="preserve">In-Store Visual Merchandising Manager_NEW </t>
+    <t>In-Store Visual Merchandising Manager_NEW </t>
   </si>
   <si>
     <t>Test_27</t>
@@ -2289,7 +2304,7 @@
     <t>94 Retail Operatives</t>
   </si>
   <si>
-    <t xml:space="preserve">01 Accessories  </t>
+    <t>01 Accessories  </t>
   </si>
   <si>
     <t>Test_31</t>
@@ -2298,7 +2313,7 @@
     <t>RATwoD</t>
   </si>
   <si>
-    <t xml:space="preserve">02 Hosiery  </t>
+    <t>02 Hosiery  </t>
   </si>
   <si>
     <t>Test_32</t>
@@ -2307,7 +2322,7 @@
     <t>RAThreeE</t>
   </si>
   <si>
-    <t xml:space="preserve">04 Lingerie  </t>
+    <t>04 Lingerie  </t>
   </si>
   <si>
     <t>Test_33</t>
@@ -2322,7 +2337,7 @@
     <t>RAFourFrerunX</t>
   </si>
   <si>
-    <t xml:space="preserve">05 Children’s Wear  </t>
+    <t>05 Children’s Wear  </t>
   </si>
   <si>
     <t>Test_34</t>
@@ -2331,7 +2346,7 @@
     <t>RAFiveG</t>
   </si>
   <si>
-    <t xml:space="preserve">06 Menswear  </t>
+    <t>06 Menswear  </t>
   </si>
   <si>
     <t>Test_35</t>
@@ -2340,7 +2355,7 @@
     <t>RASixFutH</t>
   </si>
   <si>
-    <t xml:space="preserve">07 Footwear  </t>
+    <t>07 Footwear  </t>
   </si>
   <si>
     <t>Test_36</t>
@@ -2349,7 +2364,7 @@
     <t>RASevenI</t>
   </si>
   <si>
-    <t xml:space="preserve">08 Ladieswear  </t>
+    <t>08 Ladieswear  </t>
   </si>
   <si>
     <t>Test_37</t>
@@ -2358,7 +2373,7 @@
     <t>RAEightJ</t>
   </si>
   <si>
-    <t xml:space="preserve">11 Household  </t>
+    <t>11 Household  </t>
   </si>
   <si>
     <t>Test_38</t>
@@ -2367,7 +2382,7 @@
     <t>RANineK</t>
   </si>
   <si>
-    <t xml:space="preserve">15 Children’s Accessories  </t>
+    <t>15 Children’s Accessories  </t>
   </si>
   <si>
     <t>Test_39</t>
@@ -2376,7 +2391,7 @@
     <t>RATenL</t>
   </si>
   <si>
-    <t xml:space="preserve">16 Men’s Accessories  </t>
+    <t>16 Men’s Accessories  </t>
   </si>
   <si>
     <t>Test_40</t>
@@ -2385,7 +2400,7 @@
     <t>RAElevenM</t>
   </si>
   <si>
-    <t xml:space="preserve">23 Health &amp; Beauty  </t>
+    <t>23 Health &amp; Beauty  </t>
   </si>
   <si>
     <t>Test_41</t>
@@ -2394,7 +2409,7 @@
     <t>RATwelveN</t>
   </si>
   <si>
-    <t xml:space="preserve">24 Gifts Christmas  </t>
+    <t>24 Gifts Christmas  </t>
   </si>
   <si>
     <t>Test_42</t>
@@ -2406,7 +2421,7 @@
     <t>Part Time</t>
   </si>
   <si>
-    <t xml:space="preserve">25 Primarket  </t>
+    <t>25 Primarket  </t>
   </si>
   <si>
     <t>Test_43</t>
@@ -2415,7 +2430,7 @@
     <t>RAFourteenP</t>
   </si>
   <si>
-    <t xml:space="preserve">258 Cash Office  </t>
+    <t>258 Cash Office  </t>
   </si>
   <si>
     <t>Test_44</t>
@@ -2424,7 +2439,7 @@
     <t>RAFifteenQ</t>
   </si>
   <si>
-    <t xml:space="preserve">259 Customer Service Desk  </t>
+    <t>259 Customer Service Desk  </t>
   </si>
   <si>
     <t>Test_45</t>
@@ -2433,7 +2448,7 @@
     <t>RAEighteenR</t>
   </si>
   <si>
-    <t xml:space="preserve">262 Nightshift  </t>
+    <t>262 Nightshift  </t>
   </si>
   <si>
     <t>0811111136</t>
@@ -2550,7 +2565,7 @@
     <t>RAFortyThreeI</t>
   </si>
   <si>
-    <t xml:space="preserve">260 Fitting Rooms  </t>
+    <t>260 Fitting Rooms  </t>
   </si>
   <si>
     <t>Test_63</t>
@@ -2559,7 +2574,7 @@
     <t>RAFortyFourJ</t>
   </si>
   <si>
-    <t xml:space="preserve">261 Tills  </t>
+    <t>261 Tills  </t>
   </si>
   <si>
     <t>Test_64</t>
@@ -2622,7 +2637,7 @@
     <t>RACashOneS</t>
   </si>
   <si>
-    <t xml:space="preserve">Retail Assistant Cash Office_NEW  </t>
+    <t>Retail Assistant Cash Office_NEW  </t>
   </si>
   <si>
     <t>Test_73</t>
@@ -2640,7 +2655,7 @@
     <t>RAStockOneU</t>
   </si>
   <si>
-    <t xml:space="preserve">Retail Assistant Stockroom_NEW  </t>
+    <t>Retail Assistant Stockroom_NEW  </t>
   </si>
   <si>
     <t>Test_75</t>
@@ -2667,7 +2682,7 @@
     <t>Pardubice</t>
   </si>
   <si>
-    <t xml:space="preserve">Retail Assistant Special Contracts_NEW </t>
+    <t>Retail Assistant Special Contracts_NEW </t>
   </si>
   <si>
     <t>Hourly</t>
@@ -2754,7 +2769,7 @@
     <t>PCSuperOneH</t>
   </si>
   <si>
-    <t xml:space="preserve">250 Human Resources Retail  </t>
+    <t>250 Human Resources Retail  </t>
   </si>
   <si>
     <t>Test_88</t>
@@ -2775,10 +2790,10 @@
     <t>VMOneK</t>
   </si>
   <si>
-    <t xml:space="preserve">In-Store Visual Merchandising Assistant_NEW </t>
-  </si>
-  <si>
-    <t xml:space="preserve">256 Visual Merchandising  </t>
+    <t>In-Store Visual Merchandising Assistant_NEW </t>
+  </si>
+  <si>
+    <t>256 Visual Merchandising  </t>
   </si>
   <si>
     <t>Test_91</t>
@@ -2800,16 +2815,16 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve"> </t>
+      <t> </t>
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">Operational Support_NEW  </t>
+      <t>Operational Support_NEW  </t>
     </r>
   </si>
   <si>
@@ -2843,7 +2858,7 @@
     <t>PCAssisOneS</t>
   </si>
   <si>
-    <t xml:space="preserve">In-Store P&amp;C Assistant_NEW </t>
+    <t>In-Store P&amp;C Assistant_NEW </t>
   </si>
   <si>
     <t>Test_99</t>
@@ -2873,61 +2888,61 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="14"/>
       <color rgb="FFFF0000"/>
+      <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="14"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
-    </font>
-    <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
-      <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="9">
@@ -2945,13 +2960,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.1499984740745262"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.3999755851924192"/>
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2968,13 +2983,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.0499893185216834"/>
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -2991,9 +3006,15 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -3003,15 +3024,27 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -3030,10 +3063,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -3445,14 +3484,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:CY101"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="103" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" spans="1:103" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:103" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3703,7 +3742,7 @@
       <c r="CX1" s="8"/>
       <c r="CY1" s="3"/>
     </row>
-    <row r="2" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -3817,9 +3856,9 @@
         <f t="shared" ref="AK2:AK33" si="1">L2</f>
         <v>45108</v>
       </c>
-      <c r="AL2" s="27">
+      <c r="AL2" s="27" t="str">
         <f t="shared" ref="AL2:AL33" si="2">AH2</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM2" s="28">
         <f t="shared" ref="AM2:AM33" si="3">L2</f>
@@ -3930,7 +3969,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="3" ht="14.4" customHeight="1" spans="1:73" s="34" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:103" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>114</v>
       </c>
@@ -4157,7 +4196,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="4" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>119</v>
       </c>
@@ -4271,9 +4310,9 @@
         <f t="shared" si="1"/>
         <v>44807</v>
       </c>
-      <c r="AL4" s="27">
+      <c r="AL4" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM4" s="28">
         <f t="shared" si="3"/>
@@ -4384,7 +4423,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="5" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>124</v>
       </c>
@@ -4419,8 +4458,8 @@
         <v>79</v>
       </c>
       <c r="L5" s="15">
-        <f t="shared" si="0"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45784</v>
       </c>
       <c r="M5" s="12" t="s">
         <v>74</v>
@@ -4456,8 +4495,8 @@
         <v>79</v>
       </c>
       <c r="X5" s="18">
-        <f>TODAY()+60</f>
-        <v>45769</v>
+        <f ca="1">TODAY()+60</f>
+        <v>45784</v>
       </c>
       <c r="Y5" s="14" t="s">
         <v>86</v>
@@ -4496,20 +4535,20 @@
         <v>95</v>
       </c>
       <c r="AK5" s="26">
-        <f t="shared" si="1"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45784</v>
       </c>
       <c r="AL5" s="27">
         <f t="shared" si="2"/>
         <v>46357</v>
       </c>
       <c r="AM5" s="28">
-        <f t="shared" si="3"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45784</v>
       </c>
       <c r="AN5" s="28">
-        <f t="shared" si="4"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>45784</v>
       </c>
       <c r="AO5" s="25" t="s">
         <v>96</v>
@@ -4521,8 +4560,8 @@
         <v>100</v>
       </c>
       <c r="AR5" s="28">
-        <f t="shared" si="5"/>
-        <v>45829</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>45844</v>
       </c>
       <c r="AS5" s="12" t="s">
         <v>74</v>
@@ -4612,7 +4651,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="6" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>128</v>
       </c>
@@ -4726,9 +4765,9 @@
         <f t="shared" si="1"/>
         <v>45170</v>
       </c>
-      <c r="AL6" s="27">
+      <c r="AL6" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM6" s="28">
         <f t="shared" si="3"/>
@@ -4839,7 +4878,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="7" ht="14.4" customHeight="1" spans="1:73" s="34" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:103" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>133</v>
       </c>
@@ -5066,7 +5105,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="8" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>137</v>
       </c>
@@ -5180,9 +5219,9 @@
         <f t="shared" si="1"/>
         <v>44807</v>
       </c>
-      <c r="AL8" s="27">
+      <c r="AL8" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM8" s="28">
         <f t="shared" si="3"/>
@@ -5293,7 +5332,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="9" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>141</v>
       </c>
@@ -5328,8 +5367,8 @@
         <v>79</v>
       </c>
       <c r="L9" s="15">
-        <f t="shared" si="0"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45784</v>
       </c>
       <c r="M9" s="12" t="s">
         <v>74</v>
@@ -5365,8 +5404,8 @@
         <v>79</v>
       </c>
       <c r="X9" s="18">
-        <f>TODAY()+60</f>
-        <v>45769</v>
+        <f ca="1">TODAY()+60</f>
+        <v>45784</v>
       </c>
       <c r="Y9" s="14" t="s">
         <v>86</v>
@@ -5405,20 +5444,20 @@
         <v>95</v>
       </c>
       <c r="AK9" s="26">
-        <f t="shared" si="1"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45784</v>
       </c>
       <c r="AL9" s="27">
         <f t="shared" si="2"/>
         <v>46357</v>
       </c>
       <c r="AM9" s="28">
-        <f t="shared" si="3"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45784</v>
       </c>
       <c r="AN9" s="28">
-        <f t="shared" si="4"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>45784</v>
       </c>
       <c r="AO9" s="25" t="s">
         <v>96</v>
@@ -5430,8 +5469,8 @@
         <v>100</v>
       </c>
       <c r="AR9" s="28">
-        <f t="shared" si="5"/>
-        <v>45829</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>45844</v>
       </c>
       <c r="AS9" s="12" t="s">
         <v>74</v>
@@ -5521,7 +5560,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="10" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>145</v>
       </c>
@@ -5635,9 +5674,9 @@
         <f t="shared" si="1"/>
         <v>45170</v>
       </c>
-      <c r="AL10" s="27">
+      <c r="AL10" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM10" s="28">
         <f t="shared" si="3"/>
@@ -5748,7 +5787,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="11" ht="14.4" customHeight="1" spans="1:73" s="34" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:103" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>150</v>
       </c>
@@ -5975,7 +6014,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="12" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>154</v>
       </c>
@@ -6089,9 +6128,9 @@
         <f t="shared" si="1"/>
         <v>44807</v>
       </c>
-      <c r="AL12" s="27">
+      <c r="AL12" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM12" s="28">
         <f t="shared" si="3"/>
@@ -6202,7 +6241,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="13" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>158</v>
       </c>
@@ -6237,8 +6276,8 @@
         <v>79</v>
       </c>
       <c r="L13" s="15">
-        <f t="shared" si="0"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45784</v>
       </c>
       <c r="M13" s="12" t="s">
         <v>74</v>
@@ -6274,8 +6313,8 @@
         <v>79</v>
       </c>
       <c r="X13" s="18">
-        <f>TODAY()+60</f>
-        <v>45769</v>
+        <f ca="1">TODAY()+60</f>
+        <v>45784</v>
       </c>
       <c r="Y13" s="14" t="s">
         <v>86</v>
@@ -6314,20 +6353,20 @@
         <v>95</v>
       </c>
       <c r="AK13" s="26">
-        <f t="shared" si="1"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45784</v>
       </c>
       <c r="AL13" s="27">
         <f t="shared" si="2"/>
         <v>46357</v>
       </c>
       <c r="AM13" s="28">
-        <f t="shared" si="3"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45784</v>
       </c>
       <c r="AN13" s="28">
-        <f t="shared" si="4"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>45784</v>
       </c>
       <c r="AO13" s="25" t="s">
         <v>96</v>
@@ -6339,8 +6378,8 @@
         <v>100</v>
       </c>
       <c r="AR13" s="28">
-        <f t="shared" si="5"/>
-        <v>45829</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>45844</v>
       </c>
       <c r="AS13" s="12" t="s">
         <v>74</v>
@@ -6430,7 +6469,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="14" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>162</v>
       </c>
@@ -6544,9 +6583,9 @@
         <f t="shared" si="1"/>
         <v>45170</v>
       </c>
-      <c r="AL14" s="27">
+      <c r="AL14" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM14" s="28">
         <f t="shared" si="3"/>
@@ -6657,7 +6696,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="15" ht="14.4" customHeight="1" spans="1:73" s="34" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:103" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>167</v>
       </c>
@@ -6884,7 +6923,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="16" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>171</v>
       </c>
@@ -6993,9 +7032,9 @@
         <f t="shared" si="1"/>
         <v>44807</v>
       </c>
-      <c r="AL16" s="27">
+      <c r="AL16" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM16" s="28">
         <f t="shared" si="3"/>
@@ -7106,7 +7145,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="17" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>173</v>
       </c>
@@ -7136,8 +7175,8 @@
         <v>79</v>
       </c>
       <c r="L17" s="15">
-        <f t="shared" si="0"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45784</v>
       </c>
       <c r="M17" s="12" t="s">
         <v>74</v>
@@ -7173,8 +7212,8 @@
         <v>79</v>
       </c>
       <c r="X17" s="18">
-        <f>TODAY()+60</f>
-        <v>45769</v>
+        <f ca="1">TODAY()+60</f>
+        <v>45784</v>
       </c>
       <c r="Y17" s="14" t="s">
         <v>86</v>
@@ -7213,20 +7252,20 @@
         <v>95</v>
       </c>
       <c r="AK17" s="26">
-        <f t="shared" si="1"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45784</v>
       </c>
       <c r="AL17" s="27">
         <f t="shared" si="2"/>
         <v>46357</v>
       </c>
       <c r="AM17" s="28">
-        <f t="shared" si="3"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45784</v>
       </c>
       <c r="AN17" s="28">
-        <f t="shared" si="4"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>45784</v>
       </c>
       <c r="AO17" s="25" t="s">
         <v>96</v>
@@ -7238,8 +7277,8 @@
         <v>100</v>
       </c>
       <c r="AR17" s="28">
-        <f t="shared" si="5"/>
-        <v>45829</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>45844</v>
       </c>
       <c r="AS17" s="12" t="s">
         <v>74</v>
@@ -7329,7 +7368,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="18" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>175</v>
       </c>
@@ -7438,9 +7477,9 @@
         <f t="shared" si="1"/>
         <v>45231</v>
       </c>
-      <c r="AL18" s="27">
+      <c r="AL18" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM18" s="28">
         <f t="shared" si="3"/>
@@ -7551,7 +7590,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="19" ht="14.4" customHeight="1" spans="1:73" s="34" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:73" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>178</v>
       </c>
@@ -7774,7 +7813,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="20" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>180</v>
       </c>
@@ -7883,9 +7922,9 @@
         <f t="shared" si="1"/>
         <v>44654</v>
       </c>
-      <c r="AL20" s="27">
+      <c r="AL20" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM20" s="28">
         <f t="shared" si="3"/>
@@ -7996,7 +8035,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="21" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>182</v>
       </c>
@@ -8026,8 +8065,8 @@
         <v>79</v>
       </c>
       <c r="L21" s="15">
-        <f t="shared" si="0"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45784</v>
       </c>
       <c r="M21" s="12" t="s">
         <v>74</v>
@@ -8063,8 +8102,8 @@
         <v>79</v>
       </c>
       <c r="X21" s="18">
-        <f>TODAY()+60</f>
-        <v>45769</v>
+        <f ca="1">TODAY()+60</f>
+        <v>45784</v>
       </c>
       <c r="Y21" s="14" t="s">
         <v>86</v>
@@ -8103,20 +8142,20 @@
         <v>95</v>
       </c>
       <c r="AK21" s="26">
-        <f t="shared" si="1"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45784</v>
       </c>
       <c r="AL21" s="27">
         <f t="shared" si="2"/>
         <v>46357</v>
       </c>
       <c r="AM21" s="28">
-        <f t="shared" si="3"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45784</v>
       </c>
       <c r="AN21" s="28">
-        <f t="shared" si="4"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>45784</v>
       </c>
       <c r="AO21" s="25" t="s">
         <v>96</v>
@@ -8128,8 +8167,8 @@
         <v>100</v>
       </c>
       <c r="AR21" s="28">
-        <f t="shared" si="5"/>
-        <v>45829</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>45844</v>
       </c>
       <c r="AS21" s="12" t="s">
         <v>74</v>
@@ -8219,7 +8258,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="22" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>184</v>
       </c>
@@ -8328,9 +8367,9 @@
         <f t="shared" si="1"/>
         <v>45170</v>
       </c>
-      <c r="AL22" s="27">
+      <c r="AL22" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM22" s="28">
         <f t="shared" si="3"/>
@@ -8441,7 +8480,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="23" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>188</v>
       </c>
@@ -8663,7 +8702,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="24" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>190</v>
       </c>
@@ -8772,9 +8811,9 @@
         <f t="shared" si="1"/>
         <v>44807</v>
       </c>
-      <c r="AL24" s="27">
+      <c r="AL24" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM24" s="28">
         <f t="shared" si="3"/>
@@ -8885,7 +8924,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="25" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>192</v>
       </c>
@@ -9107,7 +9146,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="26" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>194</v>
       </c>
@@ -9216,9 +9255,9 @@
         <f t="shared" si="1"/>
         <v>45170</v>
       </c>
-      <c r="AL26" s="27">
+      <c r="AL26" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM26" s="28">
         <f t="shared" si="3"/>
@@ -9329,7 +9368,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="27" ht="14.4" customHeight="1" spans="1:73" s="34" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:73" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>198</v>
       </c>
@@ -9551,7 +9590,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="28" ht="14.4" customHeight="1" spans="1:73" s="40" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:73" s="40" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>200</v>
       </c>
@@ -9773,7 +9812,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="29" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>202</v>
       </c>
@@ -9803,8 +9842,8 @@
         <v>79</v>
       </c>
       <c r="L29" s="15">
-        <f t="shared" si="0"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45784</v>
       </c>
       <c r="M29" s="12" t="s">
         <v>74</v>
@@ -9840,8 +9879,8 @@
         <v>79</v>
       </c>
       <c r="X29" s="18">
-        <f>TODAY()+60</f>
-        <v>45769</v>
+        <f ca="1">TODAY()+60</f>
+        <v>45784</v>
       </c>
       <c r="Y29" s="14" t="s">
         <v>86</v>
@@ -9880,20 +9919,20 @@
         <v>95</v>
       </c>
       <c r="AK29" s="26">
-        <f t="shared" si="1"/>
-        <v>45769</v>
-      </c>
-      <c r="AL29" s="27">
+        <f t="shared" ca="1" si="1"/>
+        <v>45784</v>
+      </c>
+      <c r="AL29" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM29" s="28">
-        <f t="shared" si="3"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45784</v>
       </c>
       <c r="AN29" s="28">
-        <f t="shared" si="4"/>
-        <v>45769</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>45784</v>
       </c>
       <c r="AO29" s="25" t="s">
         <v>96</v>
@@ -9905,8 +9944,8 @@
         <v>100</v>
       </c>
       <c r="AR29" s="28">
-        <f t="shared" si="5"/>
-        <v>45829</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>45844</v>
       </c>
       <c r="AS29" s="12" t="s">
         <v>74</v>
@@ -9996,7 +10035,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="30" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>204</v>
       </c>
@@ -10105,9 +10144,9 @@
         <f t="shared" si="1"/>
         <v>44805</v>
       </c>
-      <c r="AL30" s="27">
+      <c r="AL30" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM30" s="28">
         <f t="shared" si="3"/>
@@ -10218,7 +10257,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="31" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>211</v>
       </c>
@@ -10440,7 +10479,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="32" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>214</v>
       </c>
@@ -10549,9 +10588,9 @@
         <f t="shared" si="1"/>
         <v>44807</v>
       </c>
-      <c r="AL32" s="27">
+      <c r="AL32" s="27" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM32" s="28">
         <f t="shared" si="3"/>
@@ -10662,7 +10701,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="33" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>217</v>
       </c>
@@ -10889,7 +10928,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="34" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>221</v>
       </c>
@@ -10998,9 +11037,9 @@
         <f t="shared" ref="AK34:AK65" si="7">L34</f>
         <v>44809</v>
       </c>
-      <c r="AL34" s="27">
+      <c r="AL34" s="27" t="str">
         <f t="shared" ref="AL34:AL65" si="8">AH34</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM34" s="28">
         <f t="shared" ref="AM34:AM65" si="9">L34</f>
@@ -11111,7 +11150,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="35" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>224</v>
       </c>
@@ -11333,7 +11372,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="36" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>227</v>
       </c>
@@ -11442,9 +11481,9 @@
         <f t="shared" si="7"/>
         <v>45176</v>
       </c>
-      <c r="AL36" s="27">
+      <c r="AL36" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM36" s="28">
         <f t="shared" si="9"/>
@@ -11555,7 +11594,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="37" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>230</v>
       </c>
@@ -11777,7 +11816,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="38" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>233</v>
       </c>
@@ -11886,9 +11925,9 @@
         <f t="shared" si="7"/>
         <v>45544</v>
       </c>
-      <c r="AL38" s="27">
+      <c r="AL38" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM38" s="28">
         <f t="shared" si="9"/>
@@ -11999,7 +12038,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="39" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>236</v>
       </c>
@@ -12221,7 +12260,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="40" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>239</v>
       </c>
@@ -12330,9 +12369,9 @@
         <f t="shared" si="7"/>
         <v>44815</v>
       </c>
-      <c r="AL40" s="27">
+      <c r="AL40" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM40" s="28">
         <f t="shared" si="9"/>
@@ -12443,7 +12482,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="41" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>242</v>
       </c>
@@ -12665,7 +12704,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="42" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>245</v>
       </c>
@@ -12774,9 +12813,9 @@
         <f t="shared" si="7"/>
         <v>44908</v>
       </c>
-      <c r="AL42" s="27">
+      <c r="AL42" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM42" s="28">
         <f t="shared" si="9"/>
@@ -12887,7 +12926,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="43" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>249</v>
       </c>
@@ -13109,7 +13148,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="44" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>252</v>
       </c>
@@ -13218,9 +13257,9 @@
         <f t="shared" si="7"/>
         <v>44819</v>
       </c>
-      <c r="AL44" s="27">
+      <c r="AL44" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM44" s="28">
         <f t="shared" si="9"/>
@@ -13331,7 +13370,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="45" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>255</v>
       </c>
@@ -13553,7 +13592,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="46" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>259</v>
       </c>
@@ -13662,9 +13701,9 @@
         <f t="shared" si="7"/>
         <v>44823</v>
       </c>
-      <c r="AL46" s="27">
+      <c r="AL46" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM46" s="28">
         <f t="shared" si="9"/>
@@ -13775,7 +13814,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="47" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>261</v>
       </c>
@@ -13997,7 +14036,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="48" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>263</v>
       </c>
@@ -14106,9 +14145,9 @@
         <f t="shared" si="7"/>
         <v>44825</v>
       </c>
-      <c r="AL48" s="27">
+      <c r="AL48" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM48" s="28">
         <f t="shared" si="9"/>
@@ -14219,7 +14258,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="49" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>265</v>
       </c>
@@ -14441,7 +14480,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="50" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>268</v>
       </c>
@@ -14550,9 +14589,9 @@
         <f t="shared" si="7"/>
         <v>45102</v>
       </c>
-      <c r="AL50" s="27">
+      <c r="AL50" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM50" s="28">
         <f t="shared" si="9"/>
@@ -14663,7 +14702,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="51" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>270</v>
       </c>
@@ -14885,7 +14924,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="52" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>272</v>
       </c>
@@ -14994,9 +15033,9 @@
         <f t="shared" si="7"/>
         <v>44892</v>
       </c>
-      <c r="AL52" s="27">
+      <c r="AL52" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM52" s="28">
         <f t="shared" si="9"/>
@@ -15107,7 +15146,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="53" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>274</v>
       </c>
@@ -15329,7 +15368,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="54" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>276</v>
       </c>
@@ -15438,9 +15477,9 @@
         <f t="shared" si="7"/>
         <v>45170</v>
       </c>
-      <c r="AL54" s="27">
+      <c r="AL54" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM54" s="28">
         <f t="shared" si="9"/>
@@ -15551,7 +15590,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="55" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>278</v>
       </c>
@@ -15773,7 +15812,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="56" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>280</v>
       </c>
@@ -15882,9 +15921,9 @@
         <f t="shared" si="7"/>
         <v>44807</v>
       </c>
-      <c r="AL56" s="27">
+      <c r="AL56" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM56" s="28">
         <f t="shared" si="9"/>
@@ -15995,7 +16034,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="57" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>282</v>
       </c>
@@ -16217,7 +16256,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="58" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>285</v>
       </c>
@@ -16326,9 +16365,9 @@
         <f t="shared" si="7"/>
         <v>44811</v>
       </c>
-      <c r="AL58" s="27">
+      <c r="AL58" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM58" s="28">
         <f t="shared" si="9"/>
@@ -16439,7 +16478,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="59" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>287</v>
       </c>
@@ -16661,7 +16700,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="60" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>289</v>
       </c>
@@ -16770,9 +16809,9 @@
         <f t="shared" si="7"/>
         <v>44782</v>
       </c>
-      <c r="AL60" s="27">
+      <c r="AL60" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM60" s="28">
         <f t="shared" si="9"/>
@@ -16883,7 +16922,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="61" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>291</v>
       </c>
@@ -17105,7 +17144,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="62" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>294</v>
       </c>
@@ -17214,9 +17253,9 @@
         <f t="shared" si="7"/>
         <v>44817</v>
       </c>
-      <c r="AL62" s="27">
+      <c r="AL62" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM62" s="28">
         <f t="shared" si="9"/>
@@ -17327,7 +17366,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="63" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>297</v>
       </c>
@@ -17549,7 +17588,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="64" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>300</v>
       </c>
@@ -17658,9 +17697,9 @@
         <f t="shared" si="7"/>
         <v>44808</v>
       </c>
-      <c r="AL64" s="27">
+      <c r="AL64" s="27" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM64" s="28">
         <f t="shared" si="9"/>
@@ -17771,7 +17810,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="65" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>302</v>
       </c>
@@ -17993,7 +18032,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="66" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>305</v>
       </c>
@@ -18102,9 +18141,9 @@
         <f t="shared" ref="AK66:AK101" si="13">L66</f>
         <v>44812</v>
       </c>
-      <c r="AL66" s="27">
+      <c r="AL66" s="27" t="str">
         <f t="shared" ref="AL66:AL101" si="14">AH66</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM66" s="28">
         <f t="shared" ref="AM66:AM101" si="15">L66</f>
@@ -18215,7 +18254,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="67" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>307</v>
       </c>
@@ -18437,7 +18476,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="68" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>309</v>
       </c>
@@ -18546,9 +18585,9 @@
         <f t="shared" si="13"/>
         <v>44814</v>
       </c>
-      <c r="AL68" s="27">
+      <c r="AL68" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM68" s="28">
         <f t="shared" si="15"/>
@@ -18659,7 +18698,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="69" ht="14.4" customHeight="1" spans="1:73" s="40" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:73" s="40" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>311</v>
       </c>
@@ -18881,7 +18920,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="70" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>314</v>
       </c>
@@ -18990,9 +19029,9 @@
         <f t="shared" si="13"/>
         <v>44818</v>
       </c>
-      <c r="AL70" s="27">
+      <c r="AL70" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM70" s="28">
         <f t="shared" si="15"/>
@@ -19103,7 +19142,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="71" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>316</v>
       </c>
@@ -19325,7 +19364,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="72" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>318</v>
       </c>
@@ -19434,9 +19473,9 @@
         <f t="shared" si="13"/>
         <v>45246</v>
       </c>
-      <c r="AL72" s="27">
+      <c r="AL72" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM72" s="28">
         <f t="shared" si="15"/>
@@ -19547,7 +19586,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="73" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>321</v>
       </c>
@@ -19769,7 +19808,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="74" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>324</v>
       </c>
@@ -19878,9 +19917,9 @@
         <f t="shared" si="13"/>
         <v>44824</v>
       </c>
-      <c r="AL74" s="27">
+      <c r="AL74" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM74" s="28">
         <f t="shared" si="15"/>
@@ -19991,7 +20030,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="75" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>327</v>
       </c>
@@ -20213,7 +20252,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="76" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>329</v>
       </c>
@@ -20322,9 +20361,9 @@
         <f t="shared" si="13"/>
         <v>44826</v>
       </c>
-      <c r="AL76" s="27">
+      <c r="AL76" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM76" s="28">
         <f t="shared" si="15"/>
@@ -20435,7 +20474,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="77" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>331</v>
       </c>
@@ -20657,7 +20696,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="78" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>340</v>
       </c>
@@ -20879,7 +20918,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="79" ht="14.4" customHeight="1" spans="1:73" s="40" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:73" s="40" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>343</v>
       </c>
@@ -21101,7 +21140,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="80" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>345</v>
       </c>
@@ -21323,7 +21362,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="81" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>347</v>
       </c>
@@ -21545,7 +21584,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="82" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>349</v>
       </c>
@@ -21767,7 +21806,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="83" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>353</v>
       </c>
@@ -21989,7 +22028,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="84" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>356</v>
       </c>
@@ -22211,7 +22250,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="85" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>358</v>
       </c>
@@ -22433,7 +22472,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="86" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>360</v>
       </c>
@@ -22655,7 +22694,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="87" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>362</v>
       </c>
@@ -22764,9 +22803,9 @@
         <f t="shared" si="13"/>
         <v>44816</v>
       </c>
-      <c r="AL87" s="27">
+      <c r="AL87" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM87" s="28">
         <f t="shared" si="15"/>
@@ -22877,7 +22916,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="88" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>365</v>
       </c>
@@ -23099,7 +23138,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="89" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>367</v>
       </c>
@@ -23321,7 +23360,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="90" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>369</v>
       </c>
@@ -23430,9 +23469,9 @@
         <f t="shared" si="13"/>
         <v>45158</v>
       </c>
-      <c r="AL90" s="27">
+      <c r="AL90" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM90" s="28">
         <f t="shared" si="15"/>
@@ -23543,7 +23582,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="91" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>373</v>
       </c>
@@ -23765,7 +23804,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="92" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>375</v>
       </c>
@@ -23987,7 +24026,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="93" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>377</v>
       </c>
@@ -24209,7 +24248,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="94" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>380</v>
       </c>
@@ -24431,7 +24470,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="95" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>382</v>
       </c>
@@ -24653,7 +24692,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="96" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>384</v>
       </c>
@@ -24875,7 +24914,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="97" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>386</v>
       </c>
@@ -25097,7 +25136,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="98" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>388</v>
       </c>
@@ -25206,9 +25245,9 @@
         <f t="shared" si="13"/>
         <v>44805</v>
       </c>
-      <c r="AL98" s="27">
+      <c r="AL98" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM98" s="28">
         <f t="shared" si="15"/>
@@ -25319,7 +25358,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="99" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>391</v>
       </c>
@@ -25542,7 +25581,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="100" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>393</v>
       </c>
@@ -25769,7 +25808,7 @@
         <v>213111231</v>
       </c>
     </row>
-    <row r="101" ht="14.4" customHeight="1" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:73" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>396</v>
       </c>
@@ -25883,9 +25922,9 @@
         <f t="shared" si="13"/>
         <v>45720</v>
       </c>
-      <c r="AL101" s="27">
+      <c r="AL101" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AM101" s="28">
         <f t="shared" si="15"/>
@@ -25997,52 +26036,22 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ10:AJ101">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ10:AJ101 Y10:Y101 W10:W101 T10:T101 K10:K101 BI10:BI101" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI10:BI101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2:BI101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K10:K101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T10:T101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2:T101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W10:W101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y10:Y101">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2:Y101">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ101 Y2:Y101 W2:W101 T2:T101 K2:K101 BI2:BI101" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="V7" r:id="rId1"/>
-    <hyperlink ref="V11" r:id="rId2"/>
-    <hyperlink ref="V21" r:id="rId3"/>
-    <hyperlink ref="V23" r:id="rId4"/>
-    <hyperlink ref="V25" r:id="rId5"/>
+    <hyperlink ref="V7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="V11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="V21" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="V23" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="V25" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>